<commit_message>
Add database schema and initial settings for Sổ Lãi 60 Ngày; configure Vercel for clean URLs
</commit_message>
<xml_diff>
--- a/couple-brand/04-finance/mo-hinh-tai-chinh-60-ngay.xlsx
+++ b/couple-brand/04-finance/mo-hinh-tai-chinh-60-ngay.xlsx
@@ -27,7 +27,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="178">
   <si>
-    <t xml:space="preserve">GIẢ ĐỊNH — BI KẸO STUDIO, 60 ngày (3/11/2026 → 2/1/2027; tiền khởi động 19/10–2/11 chi 0 ₫)</t>
+    <t xml:space="preserve">GIẢ ĐỊNH — SAMESIES, 60 ngày (3/11/2026 → 2/1/2027; tiền khởi động 19/10–2/11 chi 0 ₫)</t>
   </si>
   <si>
     <t xml:space="preserve">XANH = ô nhập liệu (sửa được) · ĐEN = công thức · XANH LÁ = lấy từ sheet khác · nền VÀNG = giả định then chốt. Cột J ghi nguồn.</t>
@@ -186,25 +186,25 @@
     <t xml:space="preserve">Nguồn giá vốn</t>
   </si>
   <si>
-    <t xml:space="preserve">Áo nỉ Bi Kẹo — set 2 áo nỉ bông, in/thêu chữ cái + ngày kỷ niệm</t>
+    <t xml:space="preserve">Áo nỉ Samesies — set 2 áo nỉ bông, in/thêu chữ cái + ngày kỷ niệm</t>
   </si>
   <si>
     <t xml:space="preserve">Nỉ bông trơn 65–87k/áo: Phương Yến HCM 75–87k (MOQ 1–3), Gấu Xám HN 65–69k (MOQ 3), THIDU 68–75k → 78k ×2; in decal nhỏ 15–23k (ThunViet) hoặc thêu ≈25k/áo (CẦN BÁO GIÁ) ×2; tag + túi 6k</t>
   </si>
   <si>
-    <t xml:space="preserve">Áo thun Bi Kẹo — set 2 áo cotton 100%, in/thêu chữ cái + ngày</t>
+    <t xml:space="preserve">Áo thun Samesies — set 2 áo cotton 100%, in/thêu chữ cái + ngày</t>
   </si>
   <si>
     <t xml:space="preserve">Cotton 100%: AKUBA HCM 35–45k, Hà Đinh HN 55–65k → 50k ×2; in/thêu 25k ×2; tag + túi 6k</t>
   </si>
   <si>
-    <t xml:space="preserve">Vòng Bi Kẹo — cặp vòng titan/inox khắc tên + hộp + thiệp</t>
+    <t xml:space="preserve">Vòng Samesies — cặp vòng titan/inox khắc tên + hộp + thiệp</t>
   </si>
   <si>
     <t xml:space="preserve">Vòng tay cặp 15–17k (thitruongsi 10/2026); khắc laser ≈10k/chiếc (CẦN BÁO GIÁ); hộp lắp ráp 3,5k + thiệp 1k + túi 2,3k + sticker 1,3k</t>
   </si>
   <si>
-    <t xml:space="preserve">Hộp Quà Kỷ Niệm Bi Kẹo — áo nỉ + vòng + thiệp viết tay + hộp quà</t>
+    <t xml:space="preserve">Hộp Quà Kỷ Niệm Samesies — áo nỉ + vòng + thiệp viết tay + hộp quà</t>
   </si>
   <si>
     <t xml:space="preserve">Bằng áo nỉ (156k + 50k) + vòng (17k + 20k) + hộp quà Noel 16k + thiệp + túi 6k (Khánh Băng, thitruongsi)</t>
@@ -222,16 +222,16 @@
     <t xml:space="preserve">Khoản</t>
   </si>
   <si>
-    <t xml:space="preserve">Áo nỉ Bi Kẹo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Áo thun Bi Kẹo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vòng Bi Kẹo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hộp Quà Kỷ Niệm Bi Kẹo</t>
+    <t xml:space="preserve">Áo nỉ Samesies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Áo thun Samesies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vòng Samesies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hộp Quà Kỷ Niệm Samesies</t>
   </si>
   <si>
     <t xml:space="preserve">Đơn bình quân</t>
@@ -1669,7 +1669,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
         <v>64</v>
       </c>
@@ -2195,10 +2195,10 @@
         <v>101</v>
       </c>
       <c r="B9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="21" t="n">
         <v>1</v>
-      </c>
-      <c r="C9" s="21" t="n">
-        <v>2</v>
       </c>
       <c r="D9" s="21" t="n">
         <v>2</v>
@@ -2228,11 +2228,11 @@
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">B$5*B9</f>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C10" s="6" t="n">
         <f aca="false">C$5*C9</f>
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D10" s="6" t="n">
         <f aca="false">D$5*D9</f>
@@ -2264,7 +2264,7 @@
       </c>
       <c r="K10" s="22" t="n">
         <f aca="false">SUM(B10:J10)</f>
-        <v>166</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2273,11 +2273,11 @@
       </c>
       <c r="B11" s="18" t="n">
         <f aca="false">B10*GiaDinh!$D$32</f>
-        <v>2583378</v>
+        <v>0</v>
       </c>
       <c r="C11" s="18" t="n">
         <f aca="false">C10*GiaDinh!$D$32</f>
-        <v>5166756</v>
+        <v>2583378</v>
       </c>
       <c r="D11" s="18" t="n">
         <f aca="false">D10*GiaDinh!$D$32</f>
@@ -2309,7 +2309,7 @@
       </c>
       <c r="K11" s="16" t="n">
         <f aca="false">SUM(B11:J11)</f>
-        <v>61262964</v>
+        <v>56096208</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2318,11 +2318,11 @@
       </c>
       <c r="B12" s="18" t="n">
         <f aca="false">-B11*(GiaDinh!$B$15+GiaDinh!$C$15)</f>
-        <v>-302255.226</v>
+        <v>-0</v>
       </c>
       <c r="C12" s="18" t="n">
         <f aca="false">-C11*(GiaDinh!$B$15+GiaDinh!$C$15)</f>
-        <v>-604510.452</v>
+        <v>-302255.226</v>
       </c>
       <c r="D12" s="18" t="n">
         <f aca="false">-D11*(GiaDinh!$B$15+GiaDinh!$C$15)</f>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="K12" s="16" t="n">
         <f aca="false">SUM(B12:J12)</f>
-        <v>-7167766.788</v>
+        <v>-6563256.336</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2363,11 +2363,11 @@
       </c>
       <c r="B13" s="18" t="n">
         <f aca="false">-B11*GiaDinh!$D$15</f>
-        <v>-21312.8685</v>
+        <v>-0</v>
       </c>
       <c r="C13" s="18" t="n">
         <f aca="false">-C11*GiaDinh!$D$15</f>
-        <v>-42625.737</v>
+        <v>-21312.8685</v>
       </c>
       <c r="D13" s="18" t="n">
         <f aca="false">-D11*GiaDinh!$D$15</f>
@@ -2399,7 +2399,7 @@
       </c>
       <c r="K13" s="16" t="n">
         <f aca="false">SUM(B13:J13)</f>
-        <v>-505419.453</v>
+        <v>-462793.716</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="B14" s="18" t="n">
         <f aca="false">-B10*GiaDinh!$F$15</f>
-        <v>-13440</v>
+        <v>-0</v>
       </c>
       <c r="C14" s="18" t="n">
         <f aca="false">-C10*GiaDinh!$F$15</f>
-        <v>-26880</v>
+        <v>-13440</v>
       </c>
       <c r="D14" s="18" t="n">
         <f aca="false">-D10*GiaDinh!$F$15</f>
@@ -2444,7 +2444,7 @@
       </c>
       <c r="K14" s="16" t="n">
         <f aca="false">SUM(B14:J14)</f>
-        <v>-318720</v>
+        <v>-291840</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2453,11 +2453,11 @@
       </c>
       <c r="B15" s="18" t="n">
         <f aca="false">-B10*GiaDinh!$H$32</f>
-        <v>-1167950</v>
+        <v>-0</v>
       </c>
       <c r="C15" s="18" t="n">
         <f aca="false">-C10*GiaDinh!$H$32</f>
-        <v>-2335900</v>
+        <v>-1167950</v>
       </c>
       <c r="D15" s="18" t="n">
         <f aca="false">-D10*GiaDinh!$H$32</f>
@@ -2489,7 +2489,7 @@
       </c>
       <c r="K15" s="16" t="n">
         <f aca="false">SUM(B15:J15)</f>
-        <v>-27697100</v>
+        <v>-25361200</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2498,11 +2498,11 @@
       </c>
       <c r="B16" s="18" t="n">
         <f aca="false">-B10*(GiaDinh!$B$18+GiaDinh!$B$19)</f>
-        <v>-147000</v>
+        <v>-0</v>
       </c>
       <c r="C16" s="18" t="n">
         <f aca="false">-C10*(GiaDinh!$B$18+GiaDinh!$B$19)</f>
-        <v>-294000</v>
+        <v>-147000</v>
       </c>
       <c r="D16" s="18" t="n">
         <f aca="false">-D10*(GiaDinh!$B$18+GiaDinh!$B$19)</f>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="K16" s="16" t="n">
         <f aca="false">SUM(B16:J16)</f>
-        <v>-3486000</v>
+        <v>-3192000</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2543,11 +2543,11 @@
       </c>
       <c r="B17" s="18" t="n">
         <f aca="false">-B10*GiaDinh!$B$20*GiaDinh!$B$21</f>
-        <v>-28000</v>
+        <v>-0</v>
       </c>
       <c r="C17" s="18" t="n">
         <f aca="false">-C10*GiaDinh!$B$20*GiaDinh!$B$21</f>
-        <v>-56000</v>
+        <v>-28000</v>
       </c>
       <c r="D17" s="18" t="n">
         <f aca="false">-D10*GiaDinh!$B$20*GiaDinh!$B$21</f>
@@ -2579,7 +2579,7 @@
       </c>
       <c r="K17" s="16" t="n">
         <f aca="false">SUM(B17:J17)</f>
-        <v>-664000</v>
+        <v>-608000</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2588,11 +2588,11 @@
       </c>
       <c r="B18" s="18" t="n">
         <f aca="false">-B10*GiaDinh!$B$22</f>
-        <v>-210000</v>
+        <v>-0</v>
       </c>
       <c r="C18" s="18" t="n">
         <f aca="false">-C10*GiaDinh!$B$22</f>
-        <v>-420000</v>
+        <v>-210000</v>
       </c>
       <c r="D18" s="18" t="n">
         <f aca="false">-D10*GiaDinh!$B$22</f>
@@ -2624,7 +2624,7 @@
       </c>
       <c r="K18" s="16" t="n">
         <f aca="false">SUM(B18:J18)</f>
-        <v>-4980000</v>
+        <v>-4560000</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2678,11 +2678,11 @@
       </c>
       <c r="B20" s="16" t="n">
         <f aca="false">SUM(B11:B19)</f>
-        <v>-106580.0945</v>
+        <v>-800000</v>
       </c>
       <c r="C20" s="16" t="n">
         <f aca="false">SUM(C11:C19)</f>
-        <v>886839.811</v>
+        <v>193419.9055</v>
       </c>
       <c r="D20" s="16" t="n">
         <f aca="false">SUM(D11:D19)</f>
@@ -2714,7 +2714,7 @@
       </c>
       <c r="K20" s="16" t="n">
         <f aca="false">SUM(B20:J20)</f>
-        <v>13243957.759</v>
+        <v>11857117.948</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2723,39 +2723,39 @@
       </c>
       <c r="B21" s="18" t="n">
         <f aca="false">B20</f>
-        <v>-106580.0945</v>
+        <v>-800000</v>
       </c>
       <c r="C21" s="18" t="n">
         <f aca="false">C20+B21</f>
-        <v>780259.7165</v>
+        <v>-606580.0945</v>
       </c>
       <c r="D21" s="18" t="n">
         <f aca="false">D20+C21</f>
-        <v>1867099.5275</v>
+        <v>480259.7165</v>
       </c>
       <c r="E21" s="18" t="n">
         <f aca="false">E20+D21</f>
-        <v>3647359.244</v>
+        <v>2260519.433</v>
       </c>
       <c r="F21" s="18" t="n">
         <f aca="false">F20+E21</f>
-        <v>5327618.9605</v>
+        <v>3940779.1495</v>
       </c>
       <c r="G21" s="18" t="n">
         <f aca="false">G20+F21</f>
-        <v>7801298.5825</v>
+        <v>6414458.7715</v>
       </c>
       <c r="H21" s="18" t="n">
         <f aca="false">H20+G21</f>
-        <v>10274978.2045</v>
+        <v>8888138.3935</v>
       </c>
       <c r="I21" s="18" t="n">
         <f aca="false">I20+H21</f>
-        <v>12155237.921</v>
+        <v>10768398.11</v>
       </c>
       <c r="J21" s="18" t="n">
         <f aca="false">J20+I21</f>
-        <v>13243957.759</v>
+        <v>11857117.948</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2764,39 +2764,39 @@
       </c>
       <c r="B22" s="13" t="n">
         <f aca="false">B21/GiaDinh!$B$5</f>
-        <v>-0.00355266981666667</v>
+        <v>-0.0266666666666667</v>
       </c>
       <c r="C22" s="13" t="n">
         <f aca="false">C21/GiaDinh!$B$5</f>
-        <v>0.0260086572166667</v>
+        <v>-0.0202193364833333</v>
       </c>
       <c r="D22" s="13" t="n">
         <f aca="false">D21/GiaDinh!$B$5</f>
-        <v>0.0622366509166667</v>
+        <v>0.0160086572166667</v>
       </c>
       <c r="E22" s="13" t="n">
         <f aca="false">E21/GiaDinh!$B$5</f>
-        <v>0.121578641466667</v>
+        <v>0.0753506477666667</v>
       </c>
       <c r="F22" s="13" t="n">
         <f aca="false">F21/GiaDinh!$B$5</f>
-        <v>0.177587298683333</v>
+        <v>0.131359304983333</v>
       </c>
       <c r="G22" s="13" t="n">
         <f aca="false">G21/GiaDinh!$B$5</f>
-        <v>0.260043286083333</v>
+        <v>0.213815292383333</v>
       </c>
       <c r="H22" s="13" t="n">
         <f aca="false">H21/GiaDinh!$B$5</f>
-        <v>0.342499273483333</v>
+        <v>0.296271279783333</v>
       </c>
       <c r="I22" s="13" t="n">
         <f aca="false">I21/GiaDinh!$B$5</f>
-        <v>0.405174597366667</v>
+        <v>0.358946603666667</v>
       </c>
       <c r="J22" s="13" t="n">
         <f aca="false">J21/GiaDinh!$B$5</f>
-        <v>0.441465258633333</v>
+        <v>0.395237264933333</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2812,10 +2812,10 @@
         <v>1</v>
       </c>
       <c r="C25" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="21" t="n">
         <v>3</v>
-      </c>
-      <c r="D25" s="21" t="n">
-        <v>4</v>
       </c>
       <c r="E25" s="21" t="n">
         <v>5</v>
@@ -2846,11 +2846,11 @@
       </c>
       <c r="C26" s="6" t="n">
         <f aca="false">C$5*C25</f>
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="D26" s="6" t="n">
         <f aca="false">D$5*D25</f>
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="E26" s="6" t="n">
         <f aca="false">E$5*E25</f>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="K26" s="22" t="n">
         <f aca="false">SUM(B26:J26)</f>
-        <v>300</v>
+        <v>286</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2891,11 +2891,11 @@
       </c>
       <c r="C27" s="18" t="n">
         <f aca="false">C26*GiaDinh!$D$32</f>
-        <v>7750134</v>
+        <v>5166756</v>
       </c>
       <c r="D27" s="18" t="n">
         <f aca="false">D26*GiaDinh!$D$32</f>
-        <v>10333512</v>
+        <v>7750134</v>
       </c>
       <c r="E27" s="18" t="n">
         <f aca="false">E26*GiaDinh!$D$32</f>
@@ -2923,7 +2923,7 @@
       </c>
       <c r="K27" s="16" t="n">
         <f aca="false">SUM(B27:J27)</f>
-        <v>110716200</v>
+        <v>105549444</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2936,11 +2936,11 @@
       </c>
       <c r="C28" s="18" t="n">
         <f aca="false">-C27*(GiaDinh!$B$15+GiaDinh!$C$15)</f>
-        <v>-906765.678</v>
+        <v>-604510.452</v>
       </c>
       <c r="D28" s="18" t="n">
         <f aca="false">-D27*(GiaDinh!$B$15+GiaDinh!$C$15)</f>
-        <v>-1209020.904</v>
+        <v>-906765.678</v>
       </c>
       <c r="E28" s="18" t="n">
         <f aca="false">-E27*(GiaDinh!$B$15+GiaDinh!$C$15)</f>
@@ -2968,7 +2968,7 @@
       </c>
       <c r="K28" s="16" t="n">
         <f aca="false">SUM(B28:J28)</f>
-        <v>-12953795.4</v>
+        <v>-12349284.948</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2981,11 +2981,11 @@
       </c>
       <c r="C29" s="18" t="n">
         <f aca="false">-C27*GiaDinh!$D$15</f>
-        <v>-63938.6055</v>
+        <v>-42625.737</v>
       </c>
       <c r="D29" s="18" t="n">
         <f aca="false">-D27*GiaDinh!$D$15</f>
-        <v>-85251.474</v>
+        <v>-63938.6055</v>
       </c>
       <c r="E29" s="18" t="n">
         <f aca="false">-E27*GiaDinh!$D$15</f>
@@ -3013,7 +3013,7 @@
       </c>
       <c r="K29" s="16" t="n">
         <f aca="false">SUM(B29:J29)</f>
-        <v>-913408.65</v>
+        <v>-870782.913</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3026,11 +3026,11 @@
       </c>
       <c r="C30" s="18" t="n">
         <f aca="false">-C26*GiaDinh!$F$15</f>
-        <v>-40320</v>
+        <v>-26880</v>
       </c>
       <c r="D30" s="18" t="n">
         <f aca="false">-D26*GiaDinh!$F$15</f>
-        <v>-53760</v>
+        <v>-40320</v>
       </c>
       <c r="E30" s="18" t="n">
         <f aca="false">-E26*GiaDinh!$F$15</f>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="K30" s="16" t="n">
         <f aca="false">SUM(B30:J30)</f>
-        <v>-576000</v>
+        <v>-549120</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3071,11 +3071,11 @@
       </c>
       <c r="C31" s="18" t="n">
         <f aca="false">-C26*GiaDinh!$H$32</f>
-        <v>-3503850</v>
+        <v>-2335900</v>
       </c>
       <c r="D31" s="18" t="n">
         <f aca="false">-D26*GiaDinh!$H$32</f>
-        <v>-4671800</v>
+        <v>-3503850</v>
       </c>
       <c r="E31" s="18" t="n">
         <f aca="false">-E26*GiaDinh!$H$32</f>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="K31" s="16" t="n">
         <f aca="false">SUM(B31:J31)</f>
-        <v>-50055000</v>
+        <v>-47719100</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3116,11 +3116,11 @@
       </c>
       <c r="C32" s="18" t="n">
         <f aca="false">-C26*(GiaDinh!$B$18+GiaDinh!$B$19)</f>
-        <v>-441000</v>
+        <v>-294000</v>
       </c>
       <c r="D32" s="18" t="n">
         <f aca="false">-D26*(GiaDinh!$B$18+GiaDinh!$B$19)</f>
-        <v>-588000</v>
+        <v>-441000</v>
       </c>
       <c r="E32" s="18" t="n">
         <f aca="false">-E26*(GiaDinh!$B$18+GiaDinh!$B$19)</f>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="K32" s="16" t="n">
         <f aca="false">SUM(B32:J32)</f>
-        <v>-6300000</v>
+        <v>-6006000</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3161,11 +3161,11 @@
       </c>
       <c r="C33" s="18" t="n">
         <f aca="false">-C26*GiaDinh!$B$20*GiaDinh!$B$21</f>
-        <v>-84000</v>
+        <v>-56000</v>
       </c>
       <c r="D33" s="18" t="n">
         <f aca="false">-D26*GiaDinh!$B$20*GiaDinh!$B$21</f>
-        <v>-112000</v>
+        <v>-84000</v>
       </c>
       <c r="E33" s="18" t="n">
         <f aca="false">-E26*GiaDinh!$B$20*GiaDinh!$B$21</f>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="K33" s="16" t="n">
         <f aca="false">SUM(B33:J33)</f>
-        <v>-1200000</v>
+        <v>-1144000</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3206,11 +3206,11 @@
       </c>
       <c r="C34" s="18" t="n">
         <f aca="false">-C26*GiaDinh!$B$22</f>
-        <v>-630000</v>
+        <v>-420000</v>
       </c>
       <c r="D34" s="18" t="n">
         <f aca="false">-D26*GiaDinh!$B$22</f>
-        <v>-840000</v>
+        <v>-630000</v>
       </c>
       <c r="E34" s="18" t="n">
         <f aca="false">-E26*GiaDinh!$B$22</f>
@@ -3238,7 +3238,7 @@
       </c>
       <c r="K34" s="16" t="n">
         <f aca="false">SUM(B34:J34)</f>
-        <v>-9000000</v>
+        <v>-8580000</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3296,11 +3296,11 @@
       </c>
       <c r="C36" s="16" t="n">
         <f aca="false">SUM(C27:C35)</f>
-        <v>1580259.7165</v>
+        <v>886839.811</v>
       </c>
       <c r="D36" s="16" t="n">
         <f aca="false">SUM(D27:D35)</f>
-        <v>2473679.622</v>
+        <v>1780259.7165</v>
       </c>
       <c r="E36" s="16" t="n">
         <f aca="false">SUM(E27:E35)</f>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="K36" s="16" t="n">
         <f aca="false">SUM(B36:J36)</f>
-        <v>26517995.95</v>
+        <v>25131156.139</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3341,35 +3341,35 @@
       </c>
       <c r="C37" s="18" t="n">
         <f aca="false">C36+B37</f>
-        <v>1473679.622</v>
+        <v>780259.7165</v>
       </c>
       <c r="D37" s="18" t="n">
         <f aca="false">D36+C37</f>
-        <v>3947359.244</v>
+        <v>2560519.433</v>
       </c>
       <c r="E37" s="18" t="n">
         <f aca="false">E36+D37</f>
-        <v>7114458.7715</v>
+        <v>5727618.9605</v>
       </c>
       <c r="F37" s="18" t="n">
         <f aca="false">F36+E37</f>
-        <v>10874978.2045</v>
+        <v>9488138.3935</v>
       </c>
       <c r="G37" s="18" t="n">
         <f aca="false">G36+F37</f>
-        <v>15428917.543</v>
+        <v>14042077.732</v>
       </c>
       <c r="H37" s="18" t="n">
         <f aca="false">H36+G37</f>
-        <v>20676276.787</v>
+        <v>19289436.976</v>
       </c>
       <c r="I37" s="18" t="n">
         <f aca="false">I36+H37</f>
-        <v>24636796.22</v>
+        <v>23249956.409</v>
       </c>
       <c r="J37" s="18" t="n">
         <f aca="false">J36+I37</f>
-        <v>26517995.95</v>
+        <v>25131156.139</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3382,35 +3382,35 @@
       </c>
       <c r="C38" s="13" t="n">
         <f aca="false">C37/GiaDinh!$B$5</f>
-        <v>0.0491226540666667</v>
+        <v>0.0260086572166667</v>
       </c>
       <c r="D38" s="13" t="n">
         <f aca="false">D37/GiaDinh!$B$5</f>
-        <v>0.131578641466667</v>
+        <v>0.0853506477666667</v>
       </c>
       <c r="E38" s="13" t="n">
         <f aca="false">E37/GiaDinh!$B$5</f>
-        <v>0.237148625716667</v>
+        <v>0.190920632016667</v>
       </c>
       <c r="F38" s="13" t="n">
         <f aca="false">F37/GiaDinh!$B$5</f>
-        <v>0.362499273483333</v>
+        <v>0.316271279783333</v>
       </c>
       <c r="G38" s="13" t="n">
         <f aca="false">G37/GiaDinh!$B$5</f>
-        <v>0.514297251433333</v>
+        <v>0.468069257733333</v>
       </c>
       <c r="H38" s="13" t="n">
         <f aca="false">H37/GiaDinh!$B$5</f>
-        <v>0.689209226233333</v>
+        <v>0.642981232533333</v>
       </c>
       <c r="I38" s="13" t="n">
         <f aca="false">I37/GiaDinh!$B$5</f>
-        <v>0.821226540666667</v>
+        <v>0.774998546966667</v>
       </c>
       <c r="J38" s="13" t="n">
         <f aca="false">J37/GiaDinh!$B$5</f>
-        <v>0.883933198333333</v>
+        <v>0.837705204633333</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4058,23 +4058,23 @@
       </c>
       <c r="B58" s="6" t="n">
         <f aca="false">K10</f>
-        <v>166</v>
+        <v>152</v>
       </c>
       <c r="C58" s="18" t="n">
         <f aca="false">K11</f>
-        <v>61262964</v>
+        <v>56096208</v>
       </c>
       <c r="D58" s="16" t="n">
         <f aca="false">K20</f>
-        <v>13243957.759</v>
+        <v>11857117.948</v>
       </c>
       <c r="E58" s="13" t="n">
         <f aca="false">D58/GiaDinh!$B$5</f>
-        <v>0.441465258633333</v>
+        <v>0.395237264933333</v>
       </c>
       <c r="F58" s="3" t="str">
         <f aca="false">IF(D58&gt;=GiaDinh!$B$5,"ĐẠT KPI","Thiếu "&amp;TEXT(GiaDinh!$B$5-D58,"#,##0")&amp;" ₫")</f>
-        <v>Thiếu 16,756,042 ₫</v>
+        <v>Thiếu 18,142,882 ₫</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4083,23 +4083,23 @@
       </c>
       <c r="B59" s="6" t="n">
         <f aca="false">K26</f>
-        <v>300</v>
+        <v>286</v>
       </c>
       <c r="C59" s="18" t="n">
         <f aca="false">K27</f>
-        <v>110716200</v>
+        <v>105549444</v>
       </c>
       <c r="D59" s="16" t="n">
         <f aca="false">K36</f>
-        <v>26517995.95</v>
+        <v>25131156.139</v>
       </c>
       <c r="E59" s="13" t="n">
         <f aca="false">D59/GiaDinh!$B$5</f>
-        <v>0.883933198333333</v>
+        <v>0.837705204633333</v>
       </c>
       <c r="F59" s="3" t="str">
         <f aca="false">IF(D59&gt;=GiaDinh!$B$5,"ĐẠT KPI","Thiếu "&amp;TEXT(GiaDinh!$B$5-D59,"#,##0")&amp;" ₫")</f>
-        <v>Thiếu 3,482,004 ₫</v>
+        <v>Thiếu 4,868,844 ₫</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4210,31 +4210,31 @@
       </c>
       <c r="D5" s="18" t="n">
         <f aca="false">C12</f>
-        <v>5143147.334625</v>
+        <v>5982554.85825</v>
       </c>
       <c r="E5" s="18" t="n">
         <f aca="false">D12</f>
-        <v>5987849.5275</v>
+        <v>6165887.145625</v>
       </c>
       <c r="F5" s="18" t="n">
         <f aca="false">E12</f>
-        <v>7493921.625875</v>
+        <v>6071181.814875</v>
       </c>
       <c r="G5" s="18" t="n">
         <f aca="false">F12</f>
-        <v>9661363.62975</v>
+        <v>8238623.81875</v>
       </c>
       <c r="H5" s="18" t="n">
         <f aca="false">G12</f>
-        <v>12590175.539125</v>
+        <v>11167435.728125</v>
       </c>
       <c r="I5" s="18" t="n">
         <f aca="false">H12</f>
-        <v>16180357.354</v>
+        <v>14757617.543</v>
       </c>
       <c r="J5" s="18" t="n">
         <f aca="false">I12</f>
-        <v>23350131.64525</v>
+        <v>21927391.83425</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4247,15 +4247,15 @@
       </c>
       <c r="C6" s="19" t="n">
         <f aca="false">GiaDinh!$B$24*(KichBan!C27+KichBan!C28+KichBan!C29+KichBan!C30-KichBan!C26*GiaDinh!$B$18)+(1-GiaDinh!$B$24)*(KichBan!B27+KichBan!B28+KichBan!B29+KichBan!B30-KichBan!B26*GiaDinh!$B$18)</f>
-        <v>3201554.85825</v>
+        <v>2667962.381875</v>
       </c>
       <c r="D6" s="19" t="n">
         <f aca="false">GiaDinh!$B$24*(KichBan!D27+KichBan!D28+KichBan!D29+KichBan!D30-KichBan!D26*GiaDinh!$B$18)+(1-GiaDinh!$B$24)*(KichBan!C27+KichBan!C28+KichBan!C29+KichBan!C30-KichBan!C26*GiaDinh!$B$18)</f>
-        <v>6936702.192875</v>
+        <v>4802332.287375</v>
       </c>
       <c r="E6" s="19" t="n">
         <f aca="false">GiaDinh!$B$24*(KichBan!E27+KichBan!E28+KichBan!E29+KichBan!E30-KichBan!E26*GiaDinh!$B$18)+(1-GiaDinh!$B$24)*(KichBan!D27+KichBan!D28+KichBan!D29+KichBan!D30-KichBan!D26*GiaDinh!$B$18)</f>
-        <v>9071072.098375</v>
+        <v>7470294.66925</v>
       </c>
       <c r="F6" s="19" t="n">
         <f aca="false">GiaDinh!$B$24*(KichBan!F27+KichBan!F28+KichBan!F29+KichBan!F30-KichBan!F26*GiaDinh!$B$18)+(1-GiaDinh!$B$24)*(KichBan!E27+KichBan!E28+KichBan!E29+KichBan!E30-KichBan!E26*GiaDinh!$B$18)</f>
@@ -4279,7 +4279,7 @@
       </c>
       <c r="K6" s="16" t="n">
         <f aca="false">SUM(B6:J6)</f>
-        <v>86899346.1525</v>
+        <v>82630606.3415</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4290,10 +4290,10 @@
         <v>-2700000</v>
       </c>
       <c r="C7" s="4" t="n">
+        <v>-2400000</v>
+      </c>
+      <c r="D7" s="4" t="n">
         <v>-3500000</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>-4700000</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>-5900000</v>
@@ -4315,7 +4315,7 @@
       </c>
       <c r="K7" s="16" t="n">
         <f aca="false">SUM(B7:J7)</f>
-        <v>-51800000</v>
+        <v>-49500000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4328,11 +4328,11 @@
       </c>
       <c r="C8" s="19" t="n">
         <f aca="false">KichBan!C34</f>
-        <v>-630000</v>
+        <v>-420000</v>
       </c>
       <c r="D8" s="19" t="n">
         <f aca="false">KichBan!D34</f>
-        <v>-840000</v>
+        <v>-630000</v>
       </c>
       <c r="E8" s="19" t="n">
         <f aca="false">KichBan!E34</f>
@@ -4360,7 +4360,7 @@
       </c>
       <c r="K8" s="16" t="n">
         <f aca="false">SUM(B8:J8)</f>
-        <v>-9000000</v>
+        <v>-8580000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4373,11 +4373,11 @@
       </c>
       <c r="C9" s="19" t="n">
         <f aca="false">-KichBan!C26*GiaDinh!$B$19+KichBan!C33</f>
-        <v>-189000</v>
+        <v>-126000</v>
       </c>
       <c r="D9" s="19" t="n">
         <f aca="false">-KichBan!D26*GiaDinh!$B$19+KichBan!D33</f>
-        <v>-252000</v>
+        <v>-189000</v>
       </c>
       <c r="E9" s="19" t="n">
         <f aca="false">-KichBan!E26*GiaDinh!$B$19+KichBan!E33</f>
@@ -4405,7 +4405,7 @@
       </c>
       <c r="K9" s="16" t="n">
         <f aca="false">SUM(B9:J9)</f>
-        <v>-2700000</v>
+        <v>-2574000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4463,15 +4463,15 @@
       </c>
       <c r="C11" s="18" t="n">
         <f aca="false">SUM(C6:C10)</f>
-        <v>-1617445.14175</v>
+        <v>-778037.618125</v>
       </c>
       <c r="D11" s="18" t="n">
         <f aca="false">SUM(D6:D10)</f>
-        <v>844702.192875001</v>
+        <v>183332.287375</v>
       </c>
       <c r="E11" s="18" t="n">
         <f aca="false">SUM(E6:E10)</f>
-        <v>1506072.098375</v>
+        <v>-94705.3307499997</v>
       </c>
       <c r="F11" s="18" t="n">
         <f aca="false">SUM(F6:F10)</f>
@@ -4495,7 +4495,7 @@
       </c>
       <c r="K11" s="16" t="n">
         <f aca="false">SUM(B11:J11)</f>
-        <v>20199346.1525</v>
+        <v>18776606.3415</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4508,35 +4508,35 @@
       </c>
       <c r="C12" s="16" t="n">
         <f aca="false">C5+C11</f>
-        <v>5143147.334625</v>
+        <v>5982554.85825</v>
       </c>
       <c r="D12" s="16" t="n">
         <f aca="false">D5+D11</f>
-        <v>5987849.5275</v>
+        <v>6165887.145625</v>
       </c>
       <c r="E12" s="16" t="n">
         <f aca="false">E5+E11</f>
-        <v>7493921.625875</v>
+        <v>6071181.814875</v>
       </c>
       <c r="F12" s="16" t="n">
         <f aca="false">F5+F11</f>
-        <v>9661363.62975</v>
+        <v>8238623.81875</v>
       </c>
       <c r="G12" s="16" t="n">
         <f aca="false">G5+G11</f>
-        <v>12590175.539125</v>
+        <v>11167435.728125</v>
       </c>
       <c r="H12" s="16" t="n">
         <f aca="false">H5+H11</f>
-        <v>16180357.354</v>
+        <v>14757617.543</v>
       </c>
       <c r="I12" s="16" t="n">
         <f aca="false">I5+I11</f>
-        <v>23350131.64525</v>
+        <v>21927391.83425</v>
       </c>
       <c r="J12" s="16" t="n">
         <f aca="false">J5+J11</f>
-        <v>30199346.1525</v>
+        <v>28776606.3415</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4554,11 +4554,11 @@
       </c>
       <c r="C15" s="20" t="n">
         <f aca="false">-C7/GiaDinh!$H$32</f>
-        <v>20.9769253820797</v>
+        <v>14.3841774048547</v>
       </c>
       <c r="D15" s="20" t="n">
         <f aca="false">-D7/GiaDinh!$H$32</f>
-        <v>28.169014084507</v>
+        <v>20.9769253820797</v>
       </c>
       <c r="E15" s="20" t="n">
         <f aca="false">-E7/GiaDinh!$H$32</f>
@@ -4586,7 +4586,7 @@
       </c>
       <c r="K15" s="24" t="n">
         <f aca="false">SUM(B15:J15)</f>
-        <v>310.45849565478</v>
+        <v>296.673658975127</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4599,11 +4599,11 @@
       </c>
       <c r="C16" s="25" t="n">
         <f aca="false">KichBan!C26</f>
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="D16" s="25" t="n">
         <f aca="false">KichBan!D26</f>
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="E16" s="25" t="n">
         <f aca="false">KichBan!E26</f>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="K16" s="24" t="n">
         <f aca="false">SUM(B16:J16)</f>
-        <v>300</v>
+        <v>286</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4644,35 +4644,35 @@
       </c>
       <c r="C17" s="20" t="n">
         <f aca="false">B17+C15-C16</f>
-        <v>9.15912496254121</v>
+        <v>9.56637698531615</v>
       </c>
       <c r="D17" s="20" t="n">
         <f aca="false">C17+D15-D16</f>
-        <v>9.32813904704825</v>
+        <v>9.54330236739587</v>
       </c>
       <c r="E17" s="20" t="n">
         <f aca="false">D17+E15-E16</f>
-        <v>9.68924183398263</v>
+        <v>9.90440515433024</v>
       </c>
       <c r="F17" s="20" t="n">
         <f aca="false">E17+F15-F16</f>
-        <v>9.64309259814205</v>
+        <v>9.85825591848967</v>
       </c>
       <c r="G17" s="20" t="n">
         <f aca="false">F17+G15-G16</f>
-        <v>9.78903206472881</v>
+        <v>10.0041953850764</v>
       </c>
       <c r="H17" s="20" t="n">
         <f aca="false">G17+H15-H16</f>
-        <v>10.1270602337429</v>
+        <v>10.3422235540905</v>
       </c>
       <c r="I17" s="20" t="n">
         <f aca="false">H17+I15-I16</f>
-        <v>10.0809109979023</v>
+        <v>10.2960743182499</v>
       </c>
       <c r="J17" s="20" t="n">
         <f aca="false">I17+J15-J16</f>
-        <v>10.4584956547798</v>
+        <v>10.6736589751274</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4685,35 +4685,35 @@
       </c>
       <c r="C18" s="18" t="n">
         <f aca="false">C17*GiaDinh!$H$32</f>
-        <v>1528200</v>
+        <v>1596150</v>
       </c>
       <c r="D18" s="18" t="n">
         <f aca="false">D17*GiaDinh!$H$32</f>
-        <v>1556400</v>
+        <v>1592300</v>
       </c>
       <c r="E18" s="18" t="n">
         <f aca="false">E17*GiaDinh!$H$32</f>
-        <v>1616650</v>
+        <v>1652550</v>
       </c>
       <c r="F18" s="18" t="n">
         <f aca="false">F17*GiaDinh!$H$32</f>
-        <v>1608950</v>
+        <v>1644850</v>
       </c>
       <c r="G18" s="18" t="n">
         <f aca="false">G17*GiaDinh!$H$32</f>
-        <v>1633300</v>
+        <v>1669200</v>
       </c>
       <c r="H18" s="18" t="n">
         <f aca="false">H17*GiaDinh!$H$32</f>
-        <v>1689700</v>
+        <v>1725600</v>
       </c>
       <c r="I18" s="18" t="n">
         <f aca="false">I17*GiaDinh!$H$32</f>
-        <v>1682000</v>
+        <v>1717900</v>
       </c>
       <c r="J18" s="18" t="n">
         <f aca="false">J17*GiaDinh!$H$32</f>
-        <v>1745000</v>
+        <v>1780900</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4722,7 +4722,7 @@
       </c>
       <c r="B20" s="16" t="n">
         <f aca="false">MIN(B12:J12)</f>
-        <v>5143147.334625</v>
+        <v>5982554.85825</v>
       </c>
       <c r="C20" s="3" t="str">
         <f aca="false">IF(B20&gt;=0,"AN TOÀN: không âm vốn","CẢNH BÁO: âm tiền — giảm mua hàng/ads kỳ đó hoặc tăng cọc")</f>
@@ -4735,7 +4735,7 @@
       </c>
       <c r="B21" s="18" t="n">
         <f aca="false">J12+J18</f>
-        <v>31944346.1525</v>
+        <v>30557506.3415</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4753,11 +4753,11 @@
       </c>
       <c r="B23" s="18" t="n">
         <f aca="false">B21+B22-GiaDinh!$B$4</f>
-        <v>26517995.95</v>
+        <v>25131156.139</v>
       </c>
       <c r="C23" s="19" t="n">
         <f aca="false">KichBan!K36</f>
-        <v>26517995.95</v>
+        <v>25131156.139</v>
       </c>
       <c r="D23" s="3" t="str">
         <f aca="false">IF(ABS(B23-C23)&lt;1,"KHỚP","LỆCH")</f>
@@ -4770,7 +4770,7 @@
       </c>
       <c r="B24" s="20" t="n">
         <f aca="false">J17</f>
-        <v>10.4584956547798</v>
+        <v>10.6736589751274</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4779,11 +4779,11 @@
       </c>
       <c r="B25" s="18" t="n">
         <f aca="false">-K7</f>
-        <v>51800000</v>
+        <v>49500000</v>
       </c>
       <c r="C25" s="19" t="n">
         <f aca="false">-KichBan!K31</f>
-        <v>50055000</v>
+        <v>47719100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>